<commit_message>
atualizar front e modelo de planilha
</commit_message>
<xml_diff>
--- a/confissoes.xlsx
+++ b/confissoes.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\p-pedro.serrano\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\p-pedro.serrano\Downloads\projetocatedral1\Confissoes-Londrina\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E467716A-E8EE-4F8D-893E-9115108EAD43}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0930148F-AF01-43BC-A3B8-55ABC851F89C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{F35F436B-C307-458C-AD92-DEB104579BD9}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{F35F436B-C307-458C-AD92-DEB104579BD9}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
@@ -36,19 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="30">
-  <si>
-    <t>dia_semana</t>
-  </si>
-  <si>
-    <t>paroquia</t>
-  </si>
-  <si>
-    <t>local</t>
-  </si>
-  <si>
-    <t>horario</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="30">
   <si>
     <t>Segunda</t>
   </si>
@@ -59,18 +47,9 @@
     <t>Centro</t>
   </si>
   <si>
-    <t>14h–17h</t>
-  </si>
-  <si>
-    <t>Paróquia Nossa Senhora da Paz</t>
-  </si>
-  <si>
     <t>Bairro Alto</t>
   </si>
   <si>
-    <t>09h–11h</t>
-  </si>
-  <si>
     <t>Terça</t>
   </si>
   <si>
@@ -80,18 +59,12 @@
     <t>Vila Nova</t>
   </si>
   <si>
-    <t>15h–18h</t>
-  </si>
-  <si>
     <t>Quarta</t>
   </si>
   <si>
     <t>Paróquia Santo Antônio</t>
   </si>
   <si>
-    <t>08h–12h</t>
-  </si>
-  <si>
     <t>Quinta</t>
   </si>
   <si>
@@ -104,18 +77,12 @@
     <t>Bairro Sul</t>
   </si>
   <si>
-    <t>10h–12h</t>
-  </si>
-  <si>
     <t>Sábado</t>
   </si>
   <si>
     <t>Paróquia São João Batista</t>
   </si>
   <si>
-    <t>09h–13h</t>
-  </si>
-  <si>
     <t>Domingo</t>
   </si>
   <si>
@@ -125,14 +92,47 @@
     <t>Bairro Verde</t>
   </si>
   <si>
-    <t>08h–10h</t>
+    <t>13-14</t>
+  </si>
+  <si>
+    <t>11-12</t>
+  </si>
+  <si>
+    <t>12-18</t>
+  </si>
+  <si>
+    <t>11:30-18:40</t>
+  </si>
+  <si>
+    <t>13:00-14:00</t>
+  </si>
+  <si>
+    <t>12:00-17:00</t>
+  </si>
+  <si>
+    <t>Local</t>
+  </si>
+  <si>
+    <t>Paróquia</t>
+  </si>
+  <si>
+    <t>Seminário Xaveriano</t>
+  </si>
+  <si>
+    <t>Leste</t>
+  </si>
+  <si>
+    <t>8:00-11:00 e 14:00-17:00</t>
+  </si>
+  <si>
+    <t>Santuário Nossa Senhora de Aparecida</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -149,6 +149,15 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <u/>
       <sz val="11"/>
       <color theme="1"/>
@@ -177,7 +186,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -185,7 +194,17 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -520,135 +539,141 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{95B53A92-E13E-4D7C-A31D-5C64FD6FD9AE}">
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="3" max="9" width="8.7265625" style="5"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="29" x14ac:dyDescent="0.35">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="D1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="I1" s="7" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" ht="58" x14ac:dyDescent="0.35">
+      <c r="A2" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D2" s="4"/>
+    </row>
+    <row r="3" spans="1:9" ht="87" x14ac:dyDescent="0.35">
+      <c r="A3" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C3" s="4"/>
+      <c r="D3" s="4" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A4" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C4" s="4"/>
+      <c r="D4" s="4"/>
+      <c r="E4" s="5" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A5" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C5" s="4"/>
+      <c r="D5" s="4"/>
+    </row>
+    <row r="6" spans="1:9" ht="29" x14ac:dyDescent="0.35">
+      <c r="A6" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="B6" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" ht="29" x14ac:dyDescent="0.35">
-      <c r="A2" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" ht="58" x14ac:dyDescent="0.35">
-      <c r="A3" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A4" s="2" t="s">
+      <c r="C6" s="4"/>
+      <c r="D6" s="4"/>
+    </row>
+    <row r="7" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A7" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B7" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C4" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="D4" s="2" t="s">
+      <c r="C7" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="D7" s="4"/>
+      <c r="E7" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="G7" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="I7" s="6"/>
+    </row>
+    <row r="8" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A8" s="2" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A5" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="B5" s="2" t="s">
+      <c r="B8" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C8" s="4"/>
+      <c r="D8" s="4"/>
+      <c r="H8" s="5" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" ht="72.5" x14ac:dyDescent="0.35">
+      <c r="A9" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="C5" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D5" s="2" t="s">
+      <c r="B9" s="2" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" ht="29" x14ac:dyDescent="0.35">
-      <c r="A6" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A7" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="D7" s="2" t="s">
+      <c r="C9" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="E7" s="3"/>
-    </row>
-    <row r="8" spans="1:5" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A8" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" ht="72.5" x14ac:dyDescent="0.35">
-      <c r="A9" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>29</v>
-      </c>
+      <c r="D9" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>

</xml_diff>